<commit_message>
docs: MySQL 17 bảng, business rules, dọn MD thừa, cập nhật README
Thiết kế Database & ERD:
- docs/ERD-MYSQL.md: thiết kế MySQL 17 bảng, sơ đồ ERD Mermaid
- docs/sql/shopbike_mysql_schema.sql: CREATE TABLE đầy đủ

Business Rules:
- docs/business-rules/BUSINESS-RULES.md: toàn bộ rule có cấu trúc
- scripts/append-business-rules.mjs: append rule vào Excel
- ReBike_BusinessRules_Template.xlsx: thêm 21 rule mới

Dọn MD thừa:
- Xóa docs/ERD.md (trùng ERD-MYSQL)
- Xóa docs/VNPAY-SANDBOX-HOC-TAP.md (gộp vào PAYMENTS-VNPAY)
- Sửa ref VIETQR-MODULE → PROJECT-SUMMARY §2.7, business-rules

README:
- Bảng tài liệu docs/ theo nhóm (Tổng quan, Backend, Database, Luồng, Thanh toán, Quy tắc)
- docs/README.md: mục lục MD, thêm sql/
- Cập nhật link ERD-MYSQL, PAYMENTS-VNPAY

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/ReBike_BusinessRules_Template.xlsx
+++ b/ReBike_BusinessRules_Template.xlsx
@@ -403,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J1011"/>
+  <dimension ref="A1:J1032"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4261,13 +4261,244 @@
         <v>notificationDisplay.ts; useNotificationStore</v>
       </c>
     </row>
+    <row r="1012">
+      <c r="A1012" t="str">
+        <v>BR-ORD-01</v>
+      </c>
+      <c r="B1012" t="str">
+        <v>fulfillmentType WAREHOUSE vs DIRECT</v>
+      </c>
+      <c r="C1012" t="str">
+        <v>Order có fulfillmentType: WAREHOUSE (xe certified) hoặc DIRECT (xe unverified).</v>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="str">
+        <v>BR-ORD-02</v>
+      </c>
+      <c r="B1013" t="str">
+        <v>Luồng WAREHOUSE</v>
+      </c>
+      <c r="C1013" t="str">
+        <v>Xe tại kho → AT_WAREHOUSE_PENDING_ADMIN → admin confirm → SHIPPING (24h countdown).</v>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="str">
+        <v>BR-ORD-03</v>
+      </c>
+      <c r="B1014" t="str">
+        <v>Luồng DIRECT</v>
+      </c>
+      <c r="C1014" t="str">
+        <v>PENDING_SELLER_SHIP → seller ship-to-buyer → SHIPPING. Không qua kho.</v>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="str">
+        <v>BR-ORD-04</v>
+      </c>
+      <c r="B1015" t="str">
+        <v>Hủy đơn chỉ khi DIRECT</v>
+      </c>
+      <c r="C1015" t="str">
+        <v>Buyer chỉ hủy được khi fulfillmentType=DIRECT. WAREHOUSE không cho hủy.</v>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="str">
+        <v>BR-ORD-05</v>
+      </c>
+      <c r="B1016" t="str">
+        <v>confirm-warehouse chỉ WAREHOUSE</v>
+      </c>
+      <c r="C1016" t="str">
+        <v>Admin confirm-warehouse chỉ áp dụng đơn WAREHOUSE. DIRECT trả 400.</v>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="str">
+        <v>BR-ORD-06</v>
+      </c>
+      <c r="B1017" t="str">
+        <v>confirm-warehouse yêu cầu thanh toán</v>
+      </c>
+      <c r="C1017" t="str">
+        <v>Yêu cầu depositPaid hoặc vnpayPaymentStatus=PAID mới confirm.</v>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="str">
+        <v>BR-ORD-07</v>
+      </c>
+      <c r="B1018" t="str">
+        <v>Query đơn chờ kho</v>
+      </c>
+      <c r="C1018" t="str">
+        <v>WAREHOUSE_ONLY_FILTER: chỉ đơn fulfillmentType=WAREHOUSE.</v>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="str">
+        <v>BR-ORD-08</v>
+      </c>
+      <c r="B1019" t="str">
+        <v>Seller GET /orders</v>
+      </c>
+      <c r="C1019" t="str">
+        <v>Hai nhánh: kho (SELLER_SHIPPED, AT_WAREHOUSE, không DIRECT); direct (PENDING_SELLER_SHIP + DIRECT).</v>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="str">
+        <v>BR-ORD-09</v>
+      </c>
+      <c r="B1020" t="str">
+        <v>FIFO listing</v>
+      </c>
+      <c r="C1020" t="str">
+        <v>Available → Reserved (sau deposit) → Sold. Cancel/Fail → Available.</v>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="str">
+        <v>BR-ORD-10</v>
+      </c>
+      <c r="B1021" t="str">
+        <v>Reserve khi deposit OK</v>
+      </c>
+      <c r="C1021" t="str">
+        <v>Reserve chỉ tạo khi deposit payment thành công (24h countdown).</v>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="str">
+        <v>BR-PAY-VNP-01</v>
+      </c>
+      <c r="B1022" t="str">
+        <v>Chỉ VNPAY buyer checkout</v>
+      </c>
+      <c r="C1022" t="str">
+        <v>Bỏ CASH/COD. POST /api/buyer/orders/vnpay-checkout (DEPOSIT 8% hoặc FULL).</v>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="str">
+        <v>BR-PAY-VNP-02</v>
+      </c>
+      <c r="B1023" t="str">
+        <v>Chỉ VNPAY gói seller</v>
+      </c>
+      <c r="C1023" t="str">
+        <v>Gói đăng tin dùng VNPay (bỏ Postpay).</v>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="str">
+        <v>BR-PAY-VNP-03</v>
+      </c>
+      <c r="B1024" t="str">
+        <v>Deposit 8%</v>
+      </c>
+      <c r="C1024" t="str">
+        <v>Deposit = 8% giá trị đơn. Đồng bộ FE và BE.</v>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="str">
+        <v>BR-PAY-VNP-04</v>
+      </c>
+      <c r="B1025" t="str">
+        <v>Return URL cập nhật depositPaid</v>
+      </c>
+      <c r="C1025" t="str">
+        <v>IPN hoặc Return URL cập nhật depositPaid, vnpayPaymentStatus=PAID. Return URL cũng cập nhật khi IPN không gọi được (localhost).</v>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="str">
+        <v>BR-PAY-VNP-05</v>
+      </c>
+      <c r="B1026" t="str">
+        <v>Finalize thanh toán số dư</v>
+      </c>
+      <c r="C1026" t="str">
+        <v>Buyer thanh toán phần còn lại (khi chọn DEPOSIT) trước Complete.</v>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="str">
+        <v>BR-FIN-01</v>
+      </c>
+      <c r="B1027" t="str">
+        <v>Lấy tin từ order.listing</v>
+      </c>
+      <c r="C1027" t="str">
+        <v>Finalize ưu tiên lấy listing từ order.listing khi có orderId. Không phụ thuộc GET /bikes/:id.</v>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="str">
+        <v>BR-FIN-02</v>
+      </c>
+      <c r="B1028" t="str">
+        <v>Bỏ form địa chỉ Finalize</v>
+      </c>
+      <c r="C1028" t="str">
+        <v>Finalize không hiển thị form địa chỉ — buyer đã nhập ở checkout.</v>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="str">
+        <v>BR-FIN-03</v>
+      </c>
+      <c r="B1029" t="str">
+        <v>GET /bikes/:id chỉ PUBLISHED</v>
+      </c>
+      <c r="C1029" t="str">
+        <v>API chỉ trả PUBLISHED. RESERVED có thể 404. Finalize dùng order.listing.</v>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="str">
+        <v>BR-TIME-01</v>
+      </c>
+      <c r="B1030" t="str">
+        <v>Countdown 24h khi SHIPPING</v>
+      </c>
+      <c r="C1030" t="str">
+        <v>Hiển thị đếm ngược 24h từ expiresAt để buyer hoàn tất nhận hàng.</v>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="str">
+        <v>BR-TIME-02</v>
+      </c>
+      <c r="B1031" t="str">
+        <v>Refetch khi chờ giao</v>
+      </c>
+      <c r="C1031" t="str">
+        <v>Refetch đơn mỗi 5s khi chờ seller/kho xác nhận giao.</v>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="str">
+        <v>BR-TIME-03</v>
+      </c>
+      <c r="B1032" t="str">
+        <v>expiresAt khi chuyển SHIPPING</v>
+      </c>
+      <c r="C1032" t="str">
+        <v>Set khi admin confirm (WAREHOUSE) hoặc seller ship-to-buyer (DIRECT).</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A26:J26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J1011"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J1032"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>